<commit_message>
Bold + wrap the header row and autofit text-column widths in workbooks
Header cells are now bold with wrapped text on every sheet; string-typed
columns are width-autofit to their longest value, capped at 20 characters,
so long site names/parameter names don't blow out the sheet. Numeric/date
columns are left at the default width.
</commit_message>
<xml_diff>
--- a/data/climate/climate.xlsx
+++ b/data/climate/climate.xlsx
@@ -21,13 +21,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -50,8 +53,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,89 +425,93 @@
   </sheetPr>
   <dimension ref="A1:Q136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>huc8</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>water_year</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precip_mm</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>et_mm</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>runoff_mm</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>surf_runoff_mm</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>subsurf_runoff_mm</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>recharge_mm</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>balance_mm</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>soil_moisture_m3m3</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>snow_kgm2</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>canopy_water_kgm2</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>t2_degc</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>td2_degc</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>q2_kgkg</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>n_months</t>
         </is>
@@ -8216,49 +8226,56 @@
   </sheetPr>
   <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>huc8</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>column</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>trend</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>p_value</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>slope_per_year</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>n_years</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>significant</t>
         </is>

</xml_diff>